<commit_message>
feat(students): enforce mandatory student email and clean import template
</commit_message>
<xml_diff>
--- a/public/templates/mau-danh-sach-sinh-vien.xlsx
+++ b/public/templates/mau-danh-sach-sinh-vien.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="DanhSachSinhVien" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>MSSV</t>
   </si>
@@ -19,29 +19,32 @@
     <t>Họ Tên</t>
   </si>
   <si>
-    <t>Email (Có thể không điền, mặc định là mssv@student.hcmute.edu.vn)</t>
+    <t>Email</t>
   </si>
   <si>
     <t>Nguyễn Văn A</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>Nguyễn Văn B</t>
-  </si>
-  <si>
-    <t>nguyenvanB@gmail.com</t>
-  </si>
-  <si>
-    <t>Nguyễn Văn C</t>
+    <t>nguyenvana@gmail.com</t>
+  </si>
+  <si>
+    <t>Trần Thị B</t>
+  </si>
+  <si>
+    <t>tranthib@gmail.com</t>
+  </si>
+  <si>
+    <t>Lê Văn C</t>
+  </si>
+  <si>
+    <t>levanc@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -51,9 +54,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-    </font>
-    <font>
       <sz val="11"/>
     </font>
   </fonts>
@@ -77,12 +77,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -427,9 +424,9 @@
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="58" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -443,37 +440,37 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
-        <v>24110202</v>
-      </c>
-      <c r="B2" s="2" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>24110001</v>
+      </c>
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" ht="20" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
-        <v>24110201</v>
-      </c>
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>24110002</v>
+      </c>
+      <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
-        <v>24110200</v>
-      </c>
-      <c r="B4" s="2" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>24110003</v>
+      </c>
+      <c r="B4" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>4</v>
+      <c r="C4" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>